<commit_message>
feat: actualizar fotos reales de catalogo y activar Sea Breeze + Pomegranate 4L
- Lavaloza, Suavizante 1L/4L, Detergente 1L/4L, Guantes y Floor Cleaner
  Lime Pomegranate 1L con fotos de producto reales.
- Activa Floor Cleaner Lime Pomegranate 4L, Sea Breeze 1L y Sea Breeze 4L
  (antes Available=N, sin foto) con sus fotos reales.
- Corrige product-images.json: quita foto de Sea Breeze que estaba mal
  asociada a la galeria de Pomegranate 1L.
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restaurar selector rosado/azul en Floor Cleaner (1L y 4L)
Los Floor Cleaner no son SKUs separados por aroma: cada tamano es un
solo producto con 2 fotos (Pomegranate/Sea Breeze) para que el cliente
elija color en la misma ficha. Se habia roto al separar Sea Breeze
como productos independientes; ahora Sea Breeze 1L/4L vuelven a
Available=N y sus fotos reales quedan como segunda imagen de la
galeria de Pomegranate 1L (761796) y 4L (761741).
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -951,7 +951,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>

</xml_diff>